<commit_message>
update pokedisplay data EV10
</commit_message>
<xml_diff>
--- a/pokedisplay.xlsx
+++ b/pokedisplay.xlsx
@@ -1806,33 +1806,15 @@
       <c r="AH5" s="32">
         <v>2100.0</v>
       </c>
-      <c r="AI5" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ5" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK5" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL5" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM5" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN5" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO5" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP5" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ5" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI5" s="22"/>
+      <c r="AJ5" s="22"/>
+      <c r="AK5" s="22"/>
+      <c r="AL5" s="22"/>
+      <c r="AM5" s="22"/>
+      <c r="AN5" s="22"/>
+      <c r="AO5" s="22"/>
+      <c r="AP5" s="22"/>
+      <c r="AQ5" s="22"/>
       <c r="AR5" s="33" t="s">
         <v>40</v>
       </c>
@@ -1910,33 +1892,15 @@
       <c r="AH6" s="32">
         <v>3000.0</v>
       </c>
-      <c r="AI6" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ6" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK6" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL6" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM6" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN6" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO6" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP6" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ6" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI6" s="22"/>
+      <c r="AJ6" s="22"/>
+      <c r="AK6" s="22"/>
+      <c r="AL6" s="22"/>
+      <c r="AM6" s="22"/>
+      <c r="AN6" s="22"/>
+      <c r="AO6" s="22"/>
+      <c r="AP6" s="22"/>
+      <c r="AQ6" s="22"/>
       <c r="AR6" s="33" t="s">
         <v>44</v>
       </c>
@@ -2014,33 +1978,15 @@
       <c r="AH7" s="32">
         <v>1800.0</v>
       </c>
-      <c r="AI7" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ7" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK7" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL7" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM7" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN7" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO7" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP7" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ7" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI7" s="22"/>
+      <c r="AJ7" s="22"/>
+      <c r="AK7" s="22"/>
+      <c r="AL7" s="22"/>
+      <c r="AM7" s="22"/>
+      <c r="AN7" s="22"/>
+      <c r="AO7" s="22"/>
+      <c r="AP7" s="22"/>
+      <c r="AQ7" s="22"/>
       <c r="AR7" s="33" t="s">
         <v>48</v>
       </c>
@@ -2118,33 +2064,15 @@
       <c r="AH8" s="32">
         <v>1100.0</v>
       </c>
-      <c r="AI8" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ8" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK8" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL8" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM8" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN8" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO8" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP8" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ8" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI8" s="22"/>
+      <c r="AJ8" s="22"/>
+      <c r="AK8" s="22"/>
+      <c r="AL8" s="22"/>
+      <c r="AM8" s="22"/>
+      <c r="AN8" s="22"/>
+      <c r="AO8" s="22"/>
+      <c r="AP8" s="22"/>
+      <c r="AQ8" s="22"/>
       <c r="AR8" s="33" t="s">
         <v>52</v>
       </c>
@@ -2222,33 +2150,15 @@
       <c r="AH9" s="46">
         <v>600.0</v>
       </c>
-      <c r="AI9" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ9" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK9" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL9" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM9" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN9" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO9" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP9" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ9" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI9" s="22"/>
+      <c r="AJ9" s="22"/>
+      <c r="AK9" s="22"/>
+      <c r="AL9" s="22"/>
+      <c r="AM9" s="22"/>
+      <c r="AN9" s="22"/>
+      <c r="AO9" s="22"/>
+      <c r="AP9" s="22"/>
+      <c r="AQ9" s="22"/>
       <c r="AR9" s="33" t="s">
         <v>56</v>
       </c>
@@ -2330,33 +2240,15 @@
       <c r="AH10" s="32">
         <v>420.0</v>
       </c>
-      <c r="AI10" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ10" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK10" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL10" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM10" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN10" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO10" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP10" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ10" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI10" s="22"/>
+      <c r="AJ10" s="22"/>
+      <c r="AK10" s="22"/>
+      <c r="AL10" s="22"/>
+      <c r="AM10" s="22"/>
+      <c r="AN10" s="22"/>
+      <c r="AO10" s="22"/>
+      <c r="AP10" s="22"/>
+      <c r="AQ10" s="22"/>
       <c r="AR10" s="33" t="s">
         <v>60</v>
       </c>
@@ -2434,33 +2326,15 @@
       <c r="AH11" s="32">
         <v>1150.0</v>
       </c>
-      <c r="AI11" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ11" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK11" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL11" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM11" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN11" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO11" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP11" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ11" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI11" s="22"/>
+      <c r="AJ11" s="22"/>
+      <c r="AK11" s="22"/>
+      <c r="AL11" s="22"/>
+      <c r="AM11" s="22"/>
+      <c r="AN11" s="22"/>
+      <c r="AO11" s="22"/>
+      <c r="AP11" s="22"/>
+      <c r="AQ11" s="22"/>
       <c r="AR11" s="33" t="s">
         <v>64</v>
       </c>
@@ -2540,33 +2414,15 @@
       <c r="AH12" s="32">
         <v>580.0</v>
       </c>
-      <c r="AI12" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ12" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK12" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL12" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM12" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN12" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO12" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP12" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ12" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI12" s="22"/>
+      <c r="AJ12" s="22"/>
+      <c r="AK12" s="22"/>
+      <c r="AL12" s="22"/>
+      <c r="AM12" s="22"/>
+      <c r="AN12" s="22"/>
+      <c r="AO12" s="22"/>
+      <c r="AP12" s="22"/>
+      <c r="AQ12" s="22"/>
       <c r="AR12" s="33" t="s">
         <v>68</v>
       </c>
@@ -2646,33 +2502,15 @@
       <c r="AH13" s="32">
         <v>380.0</v>
       </c>
-      <c r="AI13" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ13" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK13" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL13" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM13" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN13" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO13" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP13" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ13" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI13" s="22"/>
+      <c r="AJ13" s="22"/>
+      <c r="AK13" s="22"/>
+      <c r="AL13" s="22"/>
+      <c r="AM13" s="22"/>
+      <c r="AN13" s="22"/>
+      <c r="AO13" s="22"/>
+      <c r="AP13" s="22"/>
+      <c r="AQ13" s="22"/>
       <c r="AR13" s="33" t="s">
         <v>72</v>
       </c>
@@ -2750,33 +2588,15 @@
       <c r="AH14" s="32">
         <v>280.0</v>
       </c>
-      <c r="AI14" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ14" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK14" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL14" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM14" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN14" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO14" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP14" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ14" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI14" s="22"/>
+      <c r="AJ14" s="22"/>
+      <c r="AK14" s="22"/>
+      <c r="AL14" s="22"/>
+      <c r="AM14" s="22"/>
+      <c r="AN14" s="22"/>
+      <c r="AO14" s="22"/>
+      <c r="AP14" s="22"/>
+      <c r="AQ14" s="22"/>
       <c r="AR14" s="33" t="s">
         <v>76</v>
       </c>
@@ -2856,33 +2676,15 @@
       <c r="AH15" s="32">
         <v>420.0</v>
       </c>
-      <c r="AI15" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ15" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK15" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL15" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM15" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN15" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO15" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP15" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ15" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI15" s="22"/>
+      <c r="AJ15" s="22"/>
+      <c r="AK15" s="22"/>
+      <c r="AL15" s="22"/>
+      <c r="AM15" s="22"/>
+      <c r="AN15" s="22"/>
+      <c r="AO15" s="22"/>
+      <c r="AP15" s="22"/>
+      <c r="AQ15" s="22"/>
       <c r="AR15" s="33" t="s">
         <v>80</v>
       </c>
@@ -2962,33 +2764,15 @@
       <c r="AH16" s="32">
         <v>330.0</v>
       </c>
-      <c r="AI16" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ16" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK16" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL16" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM16" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN16" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO16" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP16" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ16" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI16" s="22"/>
+      <c r="AJ16" s="22"/>
+      <c r="AK16" s="22"/>
+      <c r="AL16" s="22"/>
+      <c r="AM16" s="22"/>
+      <c r="AN16" s="22"/>
+      <c r="AO16" s="22"/>
+      <c r="AP16" s="22"/>
+      <c r="AQ16" s="22"/>
       <c r="AR16" s="33" t="s">
         <v>84</v>
       </c>
@@ -3070,33 +2854,15 @@
       <c r="AH17" s="32">
         <v>215.0</v>
       </c>
-      <c r="AI17" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ17" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK17" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL17" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM17" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN17" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO17" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP17" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ17" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI17" s="22"/>
+      <c r="AJ17" s="22"/>
+      <c r="AK17" s="22"/>
+      <c r="AL17" s="22"/>
+      <c r="AM17" s="22"/>
+      <c r="AN17" s="22"/>
+      <c r="AO17" s="22"/>
+      <c r="AP17" s="22"/>
+      <c r="AQ17" s="22"/>
       <c r="AR17" s="33" t="s">
         <v>90</v>
       </c>
@@ -3176,33 +2942,15 @@
       <c r="AH18" s="32">
         <v>220.0</v>
       </c>
-      <c r="AI18" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ18" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK18" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL18" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM18" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN18" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO18" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP18" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ18" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI18" s="22"/>
+      <c r="AJ18" s="22"/>
+      <c r="AK18" s="22"/>
+      <c r="AL18" s="22"/>
+      <c r="AM18" s="22"/>
+      <c r="AN18" s="22"/>
+      <c r="AO18" s="22"/>
+      <c r="AP18" s="22"/>
+      <c r="AQ18" s="22"/>
       <c r="AR18" s="33" t="s">
         <v>94</v>
       </c>
@@ -3282,33 +3030,15 @@
       <c r="AH19" s="32">
         <v>220.0</v>
       </c>
-      <c r="AI19" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ19" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK19" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL19" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM19" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN19" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO19" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP19" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ19" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI19" s="22"/>
+      <c r="AJ19" s="22"/>
+      <c r="AK19" s="22"/>
+      <c r="AL19" s="22"/>
+      <c r="AM19" s="22"/>
+      <c r="AN19" s="22"/>
+      <c r="AO19" s="22"/>
+      <c r="AP19" s="22"/>
+      <c r="AQ19" s="22"/>
       <c r="AR19" s="33" t="s">
         <v>98</v>
       </c>
@@ -3388,33 +3118,15 @@
       <c r="AH20" s="32">
         <v>245.0</v>
       </c>
-      <c r="AI20" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ20" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK20" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL20" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM20" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN20" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO20" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP20" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ20" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI20" s="22"/>
+      <c r="AJ20" s="22"/>
+      <c r="AK20" s="22"/>
+      <c r="AL20" s="22"/>
+      <c r="AM20" s="22"/>
+      <c r="AN20" s="22"/>
+      <c r="AO20" s="22"/>
+      <c r="AP20" s="22"/>
+      <c r="AQ20" s="22"/>
       <c r="AR20" s="33" t="s">
         <v>102</v>
       </c>
@@ -3498,33 +3210,15 @@
       <c r="AH21" s="32">
         <v>245.0</v>
       </c>
-      <c r="AI21" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ21" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK21" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL21" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM21" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN21" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO21" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP21" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ21" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI21" s="22"/>
+      <c r="AJ21" s="22"/>
+      <c r="AK21" s="22"/>
+      <c r="AL21" s="22"/>
+      <c r="AM21" s="22"/>
+      <c r="AN21" s="22"/>
+      <c r="AO21" s="22"/>
+      <c r="AP21" s="22"/>
+      <c r="AQ21" s="22"/>
       <c r="AR21" s="33" t="s">
         <v>106</v>
       </c>
@@ -3612,33 +3306,15 @@
       <c r="AH22" s="32">
         <v>205.0</v>
       </c>
-      <c r="AI22" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ22" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK22" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL22" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM22" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN22" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO22" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP22" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ22" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI22" s="22"/>
+      <c r="AJ22" s="22"/>
+      <c r="AK22" s="22"/>
+      <c r="AL22" s="22"/>
+      <c r="AM22" s="22"/>
+      <c r="AN22" s="22"/>
+      <c r="AO22" s="22"/>
+      <c r="AP22" s="22"/>
+      <c r="AQ22" s="22"/>
       <c r="AR22" s="33" t="s">
         <v>110</v>
       </c>
@@ -3732,33 +3408,15 @@
       <c r="AH23" s="32">
         <v>200.0</v>
       </c>
-      <c r="AI23" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ23" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK23" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL23" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM23" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN23" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO23" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP23" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ23" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI23" s="22"/>
+      <c r="AJ23" s="22"/>
+      <c r="AK23" s="22"/>
+      <c r="AL23" s="22"/>
+      <c r="AM23" s="22"/>
+      <c r="AN23" s="22"/>
+      <c r="AO23" s="22"/>
+      <c r="AP23" s="22"/>
+      <c r="AQ23" s="22"/>
       <c r="AR23" s="33" t="s">
         <v>114</v>
       </c>
@@ -3856,33 +3514,15 @@
       <c r="AH24" s="32">
         <v>210.0</v>
       </c>
-      <c r="AI24" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ24" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK24" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL24" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM24" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN24" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO24" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP24" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ24" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI24" s="22"/>
+      <c r="AJ24" s="22"/>
+      <c r="AK24" s="22"/>
+      <c r="AL24" s="22"/>
+      <c r="AM24" s="22"/>
+      <c r="AN24" s="22"/>
+      <c r="AO24" s="22"/>
+      <c r="AP24" s="22"/>
+      <c r="AQ24" s="22"/>
       <c r="AR24" s="33" t="s">
         <v>118</v>
       </c>
@@ -3990,33 +3630,15 @@
       <c r="AH25" s="32">
         <v>210.0</v>
       </c>
-      <c r="AI25" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ25" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK25" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL25" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM25" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN25" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO25" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP25" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ25" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI25" s="22"/>
+      <c r="AJ25" s="22"/>
+      <c r="AK25" s="22"/>
+      <c r="AL25" s="22"/>
+      <c r="AM25" s="22"/>
+      <c r="AN25" s="22"/>
+      <c r="AO25" s="22"/>
+      <c r="AP25" s="22"/>
+      <c r="AQ25" s="22"/>
       <c r="AR25" s="33" t="s">
         <v>122</v>
       </c>
@@ -4124,33 +3746,15 @@
       <c r="AH26" s="32">
         <v>320.0</v>
       </c>
-      <c r="AI26" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ26" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK26" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL26" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM26" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN26" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO26" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP26" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ26" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI26" s="22"/>
+      <c r="AJ26" s="22"/>
+      <c r="AK26" s="22"/>
+      <c r="AL26" s="22"/>
+      <c r="AM26" s="22"/>
+      <c r="AN26" s="22"/>
+      <c r="AO26" s="22"/>
+      <c r="AP26" s="22"/>
+      <c r="AQ26" s="22"/>
       <c r="AR26" s="33" t="s">
         <v>126</v>
       </c>
@@ -4258,33 +3862,15 @@
       <c r="AH27" s="32">
         <v>250.0</v>
       </c>
-      <c r="AI27" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ27" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK27" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL27" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM27" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN27" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO27" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP27" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ27" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI27" s="22"/>
+      <c r="AJ27" s="22"/>
+      <c r="AK27" s="22"/>
+      <c r="AL27" s="22"/>
+      <c r="AM27" s="22"/>
+      <c r="AN27" s="22"/>
+      <c r="AO27" s="22"/>
+      <c r="AP27" s="22"/>
+      <c r="AQ27" s="22"/>
       <c r="AR27" s="33" t="s">
         <v>130</v>
       </c>
@@ -4392,33 +3978,15 @@
       <c r="AH28" s="32">
         <v>230.0</v>
       </c>
-      <c r="AI28" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ28" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK28" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL28" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM28" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN28" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO28" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP28" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ28" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI28" s="22"/>
+      <c r="AJ28" s="22"/>
+      <c r="AK28" s="22"/>
+      <c r="AL28" s="22"/>
+      <c r="AM28" s="22"/>
+      <c r="AN28" s="22"/>
+      <c r="AO28" s="22"/>
+      <c r="AP28" s="22"/>
+      <c r="AQ28" s="22"/>
       <c r="AR28" s="33" t="s">
         <v>134</v>
       </c>
@@ -4526,33 +4094,15 @@
       <c r="AH29" s="32">
         <v>210.0</v>
       </c>
-      <c r="AI29" s="22">
-        <v>725.0</v>
-      </c>
-      <c r="AJ29" s="22">
-        <v>830.0</v>
-      </c>
-      <c r="AK29" s="22">
-        <v>960.0</v>
-      </c>
-      <c r="AL29" s="22">
-        <v>1320.0</v>
-      </c>
-      <c r="AM29" s="22">
-        <v>1700.0</v>
-      </c>
-      <c r="AN29" s="22">
-        <v>1450.0</v>
-      </c>
-      <c r="AO29" s="22">
-        <v>1200.0</v>
-      </c>
-      <c r="AP29" s="22">
-        <v>1800.0</v>
-      </c>
-      <c r="AQ29" s="22">
-        <v>1950.0</v>
-      </c>
+      <c r="AI29" s="22"/>
+      <c r="AJ29" s="22"/>
+      <c r="AK29" s="22"/>
+      <c r="AL29" s="22"/>
+      <c r="AM29" s="22"/>
+      <c r="AN29" s="22"/>
+      <c r="AO29" s="22"/>
+      <c r="AP29" s="22"/>
+      <c r="AQ29" s="22"/>
     </row>
     <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="4"/>

</xml_diff>